<commit_message>
Added Entity Relationship Diagram.
I have amended and updated the ERD and have uploaded it here - ready for submission.
</commit_message>
<xml_diff>
--- a/Entity Relationship Diagram.xlsx
+++ b/Entity Relationship Diagram.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1332a08b4347893b/Desktop/MSc Health Data Science/Assignment 1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1332a08b4347893b/Desktop/MSc Health Data Science/Assessment 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="250" documentId="8_{BB03E1D3-2253-4E07-811B-71B0DC0D4BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A97B38E0-D21C-4545-AF7C-A4A090612B71}"/>
+  <xr:revisionPtr revIDLastSave="262" documentId="8_{BB03E1D3-2253-4E07-811B-71B0DC0D4BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D484E30F-4259-4A4D-8503-8E1E0970D19F}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="14400" windowHeight="8170" xr2:uid="{185AF615-FE68-4665-96DF-946565C507AA}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" activeTab="1" xr2:uid="{185AF615-FE68-4665-96DF-946565C507AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Relationships" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
   <si>
     <t>Hospitals</t>
   </si>
@@ -118,75 +118,39 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Address</t>
-  </si>
-  <si>
     <t>Beds</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Accreditation</t>
   </si>
   <si>
     <t>VARCHAR(100)</t>
   </si>
   <si>
-    <t>VARCHAR(200)</t>
-  </si>
-  <si>
     <t>INT</t>
   </si>
   <si>
-    <t>VARCHAR(50)</t>
-  </si>
-  <si>
-    <t>CHAR(1)</t>
-  </si>
-  <si>
     <t>Hospital name</t>
   </si>
   <si>
-    <t>Hospital type</t>
-  </si>
-  <si>
-    <t>Street address</t>
-  </si>
-  <si>
     <t>Number of beds</t>
   </si>
   <si>
-    <t>Y/N accreditation flag</t>
-  </si>
-  <si>
-    <t>Specialty</t>
-  </si>
-  <si>
     <t>INT FOREIGN KEY</t>
   </si>
   <si>
     <t>Doctor's name</t>
   </si>
   <si>
-    <t>Area of expertise</t>
-  </si>
-  <si>
     <t>Links to Hospitals</t>
   </si>
   <si>
     <t>DOB</t>
   </si>
   <si>
-    <t>Gender</t>
-  </si>
-  <si>
     <t>DATE</t>
   </si>
   <si>
-    <t>M/F</t>
-  </si>
-  <si>
     <t>Date of birth</t>
   </si>
   <si>
@@ -233,6 +197,18 @@
   </si>
   <si>
     <t>Prescription:</t>
+  </si>
+  <si>
+    <t>VARCHAR(20)</t>
+  </si>
+  <si>
+    <t>Accreditation status</t>
+  </si>
+  <si>
+    <t>Links to Doctor</t>
+  </si>
+  <si>
+    <t>Hospital</t>
   </si>
 </sst>
 </file>
@@ -978,7 +954,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748CCEA2-EACA-4859-A214-15B31AFA5B8B}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" style="4" customWidth="1"/>
@@ -987,7 +963,7 @@
     <col min="4" max="4" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1001,9 +977,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="7" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" s="7" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>6</v>
@@ -1015,263 +991,212 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="5" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="5" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" s="5" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="7" t="s">
+    </row>
+    <row r="9" spans="1:9" s="8" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2"/>
-      <c r="B9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="5" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="J10" s="7"/>
-    </row>
-    <row r="11" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
       <c r="B11" s="5" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" s="8" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="2"/>
+      <c r="B12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" spans="1:9" s="7" customFormat="1" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-    </row>
-    <row r="13" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2"/>
-      <c r="B13" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="5" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-    </row>
-    <row r="15" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="5" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="5" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
-      <c r="I16" s="8"/>
-    </row>
-    <row r="17" spans="1:6" s="7" customFormat="1" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2"/>
+      <c r="B17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2"/>
-      <c r="B18" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="2"/>
-      <c r="B19" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="2"/>
-      <c r="B20" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-    </row>
-    <row r="21" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="2"/>
-      <c r="B21" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-    </row>
-    <row r="22" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="2"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1290,7 +1215,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -1298,46 +1223,46 @@
     </row>
     <row r="3" spans="1:4" s="9" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>